<commit_message>
feat: add guests Ali Akbar, Mohandes Anvari, Ali Akbar Behzadi and update Ghazanfar Choobin in guests list and Excel
</commit_message>
<xml_diff>
--- a/guests.xlsx
+++ b/guests.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="277">
   <si>
     <t>ردیف</t>
   </si>
@@ -832,6 +832,39 @@
   </si>
   <si>
     <t>https://panteahossein.ir/?to=amirhoseinkhosravi</t>
+  </si>
+  <si>
+    <t>جناب آقای غضنفر چوبین</t>
+  </si>
+  <si>
+    <t>aliakbar</t>
+  </si>
+  <si>
+    <t>علی اکبر عزیز</t>
+  </si>
+  <si>
+    <t>دوست حسین</t>
+  </si>
+  <si>
+    <t>https://panteahossein.ir/?to=aliakbar</t>
+  </si>
+  <si>
+    <t>anvari</t>
+  </si>
+  <si>
+    <t>جناب آقای مهندس انوری</t>
+  </si>
+  <si>
+    <t>https://panteahossein.ir/?to=anvari</t>
+  </si>
+  <si>
+    <t>behzadi</t>
+  </si>
+  <si>
+    <t>جناب آقای علی اکبر بهزادی</t>
+  </si>
+  <si>
+    <t>https://panteahossein.ir/?to=behzadi</t>
   </si>
 </sst>
 </file>
@@ -1222,7 +1255,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr defaultRowHeight="15.6" ns3:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.8984375" style="3" customWidth="1"/>
@@ -2051,7 +2084,10 @@
         <v>84</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>159</v>
+        <v>266</v>
+      </c>
+      <c r="D52" t="s">
+        <v>150</v>
       </c>
       <c r="F52" t="s">
         <v>231</v>
@@ -2615,6 +2651,54 @@
       </c>
       <c r="F86" t="s">
         <v>265</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="20.4">
+      <c r="A87" s="3">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>267</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="E87" t="s">
+        <v>269</v>
+      </c>
+      <c r="F87" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="20.4">
+      <c r="A88" s="3">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>271</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="D88" t="s">
+        <v>7</v>
+      </c>
+      <c r="F88" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="20.4">
+      <c r="A89" s="3">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>274</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="F89" t="s">
+        <v>276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add guest Hojjat Farahbakhsh to guests list and Excel
</commit_message>
<xml_diff>
--- a/guests.xlsx
+++ b/guests.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="281">
   <si>
     <t>ردیف</t>
   </si>
@@ -865,6 +865,18 @@
   </si>
   <si>
     <t>https://panteahossein.ir/?to=behzadi</t>
+  </si>
+  <si>
+    <t>hojjat-farahbakhsh</t>
+  </si>
+  <si>
+    <t>جناب آقای حجت الله فرحبخش</t>
+  </si>
+  <si>
+    <t>همسر محترم</t>
+  </si>
+  <si>
+    <t>https://panteahossein.ir/?to=hojjat-farahbakhsh</t>
   </si>
 </sst>
 </file>
@@ -1255,7 +1267,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr defaultRowHeight="15.6" ns3:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.8984375" style="3" customWidth="1"/>
@@ -2701,6 +2713,23 @@
         <v>276</v>
       </c>
     </row>
+    <row r="90" spans="1:6" ht="20.4">
+      <c r="A90" s="3">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>277</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="D90" t="s">
+        <v>279</v>
+      </c>
+      <c r="F90" t="s">
+        <v>280</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
fix: update companions for Hojjat Farahbakhsh to با همسر محترم
</commit_message>
<xml_diff>
--- a/guests.xlsx
+++ b/guests.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="282">
   <si>
     <t>ردیف</t>
   </si>
@@ -877,6 +877,9 @@
   </si>
   <si>
     <t>https://panteahossein.ir/?to=hojjat-farahbakhsh</t>
+  </si>
+  <si>
+    <t>با همسر محترم</t>
   </si>
 </sst>
 </file>
@@ -2724,7 +2727,7 @@
         <v>278</v>
       </c>
       <c r="D90" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="F90" t="s">
         <v>280</v>

</xml_diff>